<commit_message>
Add SOH report for 2026-10-14
</commit_message>
<xml_diff>
--- a/reports/SOH_13_10_2026.xlsx
+++ b/reports/SOH_13_10_2026.xlsx
@@ -6817,7 +6817,7 @@
         </is>
       </c>
       <c r="D231" s="2" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E231" s="3" t="n">
         <v>1</v>
@@ -6873,7 +6873,7 @@
         </is>
       </c>
       <c r="D233" s="2" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E233" s="3" t="n">
         <v>1</v>
@@ -9626,7 +9626,7 @@
         </is>
       </c>
       <c r="D332" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E332" s="3" t="n">
         <v>5000</v>
@@ -15730,7 +15730,7 @@
         </is>
       </c>
       <c r="D550" s="2" t="n">
-        <v>312</v>
+        <v>372</v>
       </c>
       <c r="E550" s="3" t="n">
         <v>13522</v>

</xml_diff>